<commit_message>
Expand spring catalog for March and May
</commit_message>
<xml_diff>
--- a/cz_rostliny_rozsireny_dataset_v6_jadro_bezne_trvanlive.xlsx
+++ b/cz_rostliny_rozsireny_dataset_v6_jadro_bezne_trvanlive.xlsx
@@ -983,7 +983,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y257"/>
+  <dimension ref="A1:Y274"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -30375,7 +30375,6 @@
           <t>Sbírat jen opravdu mladé listy; starší rychle tuhnou a ztrácejí kulinární kvalitu.</t>
         </is>
       </c>
-      <c r="S239" t="inlineStr"/>
       <c r="T239" t="inlineStr">
         <is>
           <t>Běžný nechráněný druh; netrhat ve velkém z mladých semenáčků a v chráněných územích respektovat místní režim.</t>
@@ -30396,7 +30395,6 @@
           <t>S79</t>
         </is>
       </c>
-      <c r="X239" t="inlineStr"/>
       <c r="Y239" t="inlineStr">
         <is>
           <t>Dubnové rozšíření repertoáru o jemnou lesní listovou zeleninu.</t>
@@ -30519,7 +30517,6 @@
           <t>S80</t>
         </is>
       </c>
-      <c r="X240" t="inlineStr"/>
       <c r="Y240" t="inlineStr">
         <is>
           <t>Rozšíření dubna o jedlou jarní část hlohu, ne jen plody a EMA drogu.</t>
@@ -30642,7 +30639,6 @@
           <t>S80</t>
         </is>
       </c>
-      <c r="X241" t="inlineStr"/>
       <c r="Y241" t="inlineStr">
         <is>
           <t>Doplňuje dubnové použití hlohu i o trvanlivou formu.</t>
@@ -30765,7 +30761,6 @@
           <t>S81</t>
         </is>
       </c>
-      <c r="X242" t="inlineStr"/>
       <c r="Y242" t="inlineStr">
         <is>
           <t>Nový dubnový druh se silnou sezónností vlhkých luk.</t>
@@ -30888,7 +30883,6 @@
           <t>S82</t>
         </is>
       </c>
-      <c r="X243" t="inlineStr"/>
       <c r="Y243" t="inlineStr">
         <is>
           <t>Dubnové rozšíření se silným přesahem do dlouhodobého kuchyňského zpracování.</t>
@@ -30986,7 +30980,6 @@
           <t>Starší listy rychle tuhnou a ztrácejí kvalitu; nesbírat z prašných uličních stromů.</t>
         </is>
       </c>
-      <c r="S244" t="inlineStr"/>
       <c r="T244" t="inlineStr">
         <is>
           <t>Běžný nechráněný druh; sbírat střídmě a nepoškozovat mladé výhony ani uliční stromořadí.</t>
@@ -31007,7 +31000,6 @@
           <t>S83</t>
         </is>
       </c>
-      <c r="X244" t="inlineStr"/>
       <c r="Y244" t="inlineStr">
         <is>
           <t>Rozšiřuje duben o velmi použitelnou, ale málo zmiňovanou stromovou zeleninu.</t>
@@ -31105,7 +31097,6 @@
           <t>Nenavrtávat veřejné ani cizí stromy; odběr může strom poškodit a výtěžnost bývá nízká.</t>
         </is>
       </c>
-      <c r="S245" t="inlineStr"/>
       <c r="T245" t="inlineStr">
         <is>
           <t>Pouze na vlastních stromech nebo se souhlasem správce; v krajině nepoškozovat kmeny ani silnější větve.</t>
@@ -31126,7 +31117,6 @@
           <t>S83</t>
         </is>
       </c>
-      <c r="X245" t="inlineStr"/>
       <c r="Y245" t="inlineStr">
         <is>
           <t>Zařazeno jako dubnová niche znalost s explicitním důrazem na šetrnost odběru.</t>
@@ -31224,7 +31214,6 @@
           <t>Starší listy bývají chlupaté a méně příjemné; sbírat jen bezpečně určený plicník na čistém stanovišti.</t>
         </is>
       </c>
-      <c r="S246" t="inlineStr"/>
       <c r="T246" t="inlineStr">
         <is>
           <t>Sbírat jen jednotlivé listy tam, kde je druh běžný, a ne z chemicky ošetřovaných okrasných výsadeb.</t>
@@ -31245,7 +31234,6 @@
           <t>S84</t>
         </is>
       </c>
-      <c r="X246" t="inlineStr"/>
       <c r="Y246" t="inlineStr">
         <is>
           <t>Vědomě přidaný tajnější dubnový druh mimo běžné foragerské seznamy.</t>
@@ -31368,7 +31356,6 @@
           <t>S85</t>
         </is>
       </c>
-      <c r="X247" t="inlineStr"/>
       <c r="Y247" t="inlineStr">
         <is>
           <t>Přidává velmi časnou a snadno dostupnou dubnovou řeřišnicovou chuť.</t>
@@ -31466,7 +31453,6 @@
           <t>Největší riziko je kontaminace vody; nesbírat z odvodňovacích struh, kanalizačních přítoků ani stojatých znečištěných vod.</t>
         </is>
       </c>
-      <c r="S248" t="inlineStr"/>
       <c r="T248" t="inlineStr">
         <is>
           <t>Sbírat jen malé množství a jen z čistých lokalit bez poškozování mokřadního stanoviště.</t>
@@ -31487,7 +31473,6 @@
           <t>S86</t>
         </is>
       </c>
-      <c r="X248" t="inlineStr"/>
       <c r="Y248" t="inlineStr">
         <is>
           <t>Zařazeno schválně jako niche mokřadní jedlá rostlina s vysokým důrazem na hygienu stanoviště.</t>
@@ -31585,7 +31570,6 @@
           <t>Vysoké riziko záměny s prudce jedovatými miříkovitými; bez odborné jistoty nesbírat vůbec.</t>
         </is>
       </c>
-      <c r="S249" t="inlineStr"/>
       <c r="T249" t="inlineStr">
         <is>
           <t>Běžný nechráněný druh, ale prakticky jen pro sběrače s velmi dobrou znalostí čeledi Apiaceae.</t>
@@ -31606,7 +31590,6 @@
           <t>S87</t>
         </is>
       </c>
-      <c r="X249" t="inlineStr"/>
       <c r="Y249" t="inlineStr">
         <is>
           <t>Přidané záměrně jako pokročilejší a rizikovější dubnová položka se silným varováním.</t>
@@ -31704,7 +31687,6 @@
           <t>Sběr má smysl jen v krátkém okně mladých listů a mimo silně znečištěná stanoviště.</t>
         </is>
       </c>
-      <c r="S250" t="inlineStr"/>
       <c r="T250" t="inlineStr">
         <is>
           <t>Sbírat střídmě jednotlivé listy a nepoškozovat mladé stromky ani výsadby.</t>
@@ -31725,7 +31707,6 @@
           <t>S88</t>
         </is>
       </c>
-      <c r="X250" t="inlineStr"/>
       <c r="Y250" t="inlineStr">
         <is>
           <t>Rozšíření o další stromovou jedlost, tentokrát z výrazně okrajové znalostní vrstvy.</t>
@@ -31848,7 +31829,6 @@
           <t>S89</t>
         </is>
       </c>
-      <c r="X251" t="inlineStr"/>
       <c r="Y251" t="inlineStr">
         <is>
           <t>Záměrně přidáno jako málo známá dubnová brukvovitá alternativa mimo mainstreamové seznamy.</t>
@@ -31946,7 +31926,6 @@
           <t>Sbírat jen z čistých míst mimo psí zóny, okraje silnic a chemicky ošetřené plochy.</t>
         </is>
       </c>
-      <c r="S252" t="inlineStr"/>
       <c r="T252" t="inlineStr">
         <is>
           <t>Velmi běžný nechráněný druh; vhodný hlavně ze zahradních a jinak čistých stanovišť.</t>
@@ -31967,7 +31946,6 @@
           <t>S90</t>
         </is>
       </c>
-      <c r="X252" t="inlineStr"/>
       <c r="Y252" t="inlineStr">
         <is>
           <t>Ultra-niche dubnová položka zaměřená na nenápadné městské a lemové jedlosti.</t>
@@ -32090,7 +32068,6 @@
           <t>S91</t>
         </is>
       </c>
-      <c r="X253" t="inlineStr"/>
       <c r="Y253" t="inlineStr">
         <is>
           <t>Ultra-niche dubnový brukvovitý list s ostřejší chutí než řeřišničník.</t>
@@ -32188,7 +32165,6 @@
           <t>Preferovat sběr z vlastních nebo známých neošetřených výsadeb; okrasné rostliny mohou být chemicky ošetřené.</t>
         </is>
       </c>
-      <c r="S254" t="inlineStr"/>
       <c r="T254" t="inlineStr">
         <is>
           <t>Prakticky nejbezpečnější je sběr z vlastních výsadeb nebo legálně přístupných zplaňujících porostů.</t>
@@ -32209,7 +32185,6 @@
           <t>S92</t>
         </is>
       </c>
-      <c r="X254" t="inlineStr"/>
       <c r="Y254" t="inlineStr">
         <is>
           <t>Ultra-niche dubnová položka propojující jedlou zahradu a zplaňující flóru.</t>
@@ -32307,7 +32282,6 @@
           <t>Sbírat jen bezpečně určený zvonek a ne z okrasných výsadeb ošetřených postřiky.</t>
         </is>
       </c>
-      <c r="S255" t="inlineStr"/>
       <c r="T255" t="inlineStr">
         <is>
           <t>Lokálně běžný nechráněný druh; sbírat střídmě a nevytrhávat celé rostliny.</t>
@@ -32328,7 +32302,6 @@
           <t>S93</t>
         </is>
       </c>
-      <c r="X255" t="inlineStr"/>
       <c r="Y255" t="inlineStr">
         <is>
           <t>Ultra-niche dubnová položka pro uživatele, kteří chtějí překročit běžný seznam jarních zelení.</t>
@@ -32451,7 +32424,6 @@
           <t>S94</t>
         </is>
       </c>
-      <c r="X256" t="inlineStr"/>
       <c r="Y256" t="inlineStr">
         <is>
           <t>Ultra-niche dubnová řeřichová alternativa mimo běžný domácí repertoár.</t>
@@ -32549,7 +32521,6 @@
           <t>Sbírat jen mladé listy a jen při jistém určení; starší listy jsou tužší a méně vhodné.</t>
         </is>
       </c>
-      <c r="S257" t="inlineStr"/>
       <c r="T257" t="inlineStr">
         <is>
           <t>Lokálně běžný nechráněný druh; sbírat po jednotlivých listech a nevytrhávat celé rostliny.</t>
@@ -32570,10 +32541,2080 @@
           <t>S95</t>
         </is>
       </c>
-      <c r="X257" t="inlineStr"/>
       <c r="Y257" t="inlineStr">
         <is>
           <t>Ultra-niche dubnový doplněk pro hlubší, regionálněji znějící repertoár.</t>
+        </is>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" t="inlineStr">
+        <is>
+          <t>R257</t>
+        </is>
+      </c>
+      <c r="B258" t="inlineStr">
+        <is>
+          <t>Tussilago farfara</t>
+        </is>
+      </c>
+      <c r="C258" t="inlineStr">
+        <is>
+          <t>podběl lékařský</t>
+        </is>
+      </c>
+      <c r="D258" t="inlineStr">
+        <is>
+          <t>původní, běžný</t>
+        </is>
+      </c>
+      <c r="E258" t="inlineStr">
+        <is>
+          <t>květní poupata a mladé květy</t>
+        </is>
+      </c>
+      <c r="F258" t="inlineStr">
+        <is>
+          <t>potrava</t>
+        </is>
+      </c>
+      <c r="G258" t="inlineStr">
+        <is>
+          <t>časná květní poupata a květy do salátu / krátce tepelně</t>
+        </is>
+      </c>
+      <c r="H258" t="inlineStr">
+        <is>
+          <t>téměř zapomenuté</t>
+        </is>
+      </c>
+      <c r="I258" t="inlineStr">
+        <is>
+          <t>střední</t>
+        </is>
+      </c>
+      <c r="J258" t="inlineStr">
+        <is>
+          <t>jílovité náspy, okraje cest, výsypky, rumiště, vlhčí svahy a narušené půdy</t>
+        </is>
+      </c>
+      <c r="K258" t="inlineStr">
+        <is>
+          <t>III–IV</t>
+        </is>
+      </c>
+      <c r="L258" t="inlineStr">
+        <is>
+          <t>čerstvě vyrašené květní stvoly a polootvřená poupata před plným rozkvětem</t>
+        </is>
+      </c>
+      <c r="M258" t="inlineStr">
+        <is>
+          <t>Sbírat jen malé množství mladých květních poupat a čerstvých květů, použít je syrové jako aromatický detail do jarní směsi nebo je krátce tepelně upravit.</t>
+        </is>
+      </c>
+      <c r="N258" t="inlineStr">
+        <is>
+          <t>Velmi raná, aromatická jarní květní jedlost, která posouvá sběr až do opravdu předjarního období.</t>
+        </is>
+      </c>
+      <c r="O258" t="inlineStr">
+        <is>
+          <t>lehce anýzová, nahořkle aromatická</t>
+        </is>
+      </c>
+      <c r="P258" t="inlineStr">
+        <is>
+          <t>jemně lékořicový, květní</t>
+        </is>
+      </c>
+      <c r="Q258" t="inlineStr">
+        <is>
+          <t>neaplikovatelné</t>
+        </is>
+      </c>
+      <c r="R258" t="inlineStr">
+        <is>
+          <t>Rostlina obsahuje pyrrolizidinové alkaloidy; nejde o každodenní potravinu a sběr z krajnic nebo znečištěných náspů je nevhodný.</t>
+        </is>
+      </c>
+      <c r="S258" t="inlineStr">
+        <is>
+          <t>Nevhodné v těhotenství, při kojení a pro malé děti; nepoužívat dlouhodobě ani ve velkém množství.</t>
+        </is>
+      </c>
+      <c r="T258" t="inlineStr">
+        <is>
+          <t>Sbírat jen malé množství mimo chráněné lokality a mimo dopravně či chemicky zatížená místa.</t>
+        </is>
+      </c>
+      <c r="U258" t="inlineStr">
+        <is>
+          <t>kurátorovaný botanický zdroj</t>
+        </is>
+      </c>
+      <c r="V258" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="W258" t="inlineStr">
+        <is>
+          <t>S96</t>
+        </is>
+      </c>
+      <c r="X258" t="inlineStr"/>
+      <c r="Y258" t="inlineStr">
+        <is>
+          <t>Březnová květní vlna záměrně přidává i málo využívané předjarní druhy s opatrným rámováním rizik.</t>
+        </is>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" t="inlineStr">
+        <is>
+          <t>R258</t>
+        </is>
+      </c>
+      <c r="B259" t="inlineStr">
+        <is>
+          <t>Tussilago farfara</t>
+        </is>
+      </c>
+      <c r="C259" t="inlineStr">
+        <is>
+          <t>podběl lékařský</t>
+        </is>
+      </c>
+      <c r="D259" t="inlineStr">
+        <is>
+          <t>původní, běžný</t>
+        </is>
+      </c>
+      <c r="E259" t="inlineStr">
+        <is>
+          <t>listy a květy</t>
+        </is>
+      </c>
+      <c r="F259" t="inlineStr">
+        <is>
+          <t>pití</t>
+        </is>
+      </c>
+      <c r="G259" t="inlineStr">
+        <is>
+          <t>sušené listy a květy na občasný nálev</t>
+        </is>
+      </c>
+      <c r="H259" t="inlineStr">
+        <is>
+          <t>téměř zapomenuté</t>
+        </is>
+      </c>
+      <c r="I259" t="inlineStr">
+        <is>
+          <t>nízká až střední</t>
+        </is>
+      </c>
+      <c r="J259" t="inlineStr">
+        <is>
+          <t>jílovité náspy, okraje cest, výsypky, rumiště, vlhčí svahy a narušené půdy</t>
+        </is>
+      </c>
+      <c r="K259" t="inlineStr">
+        <is>
+          <t>III–V + sušení</t>
+        </is>
+      </c>
+      <c r="L259" t="inlineStr">
+        <is>
+          <t>časné květy a později mladší listy sbírané jen z čistých míst</t>
+        </is>
+      </c>
+      <c r="M259" t="inlineStr">
+        <is>
+          <t>Květy a mladší listy šetrně usušit a pak je používat jen střídmě a občas do lehkého bylinného nálevu.</t>
+        </is>
+      </c>
+      <c r="N259" t="inlineStr">
+        <is>
+          <t>Historizující jarní čajová surovina s jemně lékořicovým profilem, ale nízkou praktickou prioritou kvůli rizikům.</t>
+        </is>
+      </c>
+      <c r="O259" t="inlineStr">
+        <is>
+          <t>bylinná, lehce nahořklá, s nádechem lékořice</t>
+        </is>
+      </c>
+      <c r="P259" t="inlineStr">
+        <is>
+          <t>jemně květní a bylinný</t>
+        </is>
+      </c>
+      <c r="Q259" t="inlineStr">
+        <is>
+          <t>neaplikovatelné</t>
+        </is>
+      </c>
+      <c r="R259" t="inlineStr">
+        <is>
+          <t>Kvůli pyrrolizidinovým alkaloidům má dávat smysl jen občasné a střídmé použití; ne pro děti a ne dlouhodobě.</t>
+        </is>
+      </c>
+      <c r="S259" t="inlineStr">
+        <is>
+          <t>Nevhodné v těhotenství, při kojení, u malých dětí a pro dlouhodobé pravidelné pití.</t>
+        </is>
+      </c>
+      <c r="T259" t="inlineStr">
+        <is>
+          <t>Sbírat jen v malém, mimo chráněná území a mimo dopravně či chemicky zatížené lokality.</t>
+        </is>
+      </c>
+      <c r="U259" t="inlineStr">
+        <is>
+          <t>kurátorovaný botanický zdroj</t>
+        </is>
+      </c>
+      <c r="V259" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="W259" t="inlineStr">
+        <is>
+          <t>S96</t>
+        </is>
+      </c>
+      <c r="X259" t="inlineStr"/>
+      <c r="Y259" t="inlineStr">
+        <is>
+          <t>Zařazeno jako březnový trvanlivější relikt tradičního využití, ale vědomě mimo doporučený výběr.</t>
+        </is>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" t="inlineStr">
+        <is>
+          <t>R259</t>
+        </is>
+      </c>
+      <c r="B260" t="inlineStr">
+        <is>
+          <t>Primula elatior</t>
+        </is>
+      </c>
+      <c r="C260" t="inlineStr">
+        <is>
+          <t>prvosenka vyšší</t>
+        </is>
+      </c>
+      <c r="D260" t="inlineStr">
+        <is>
+          <t>původní, lokálně běžná</t>
+        </is>
+      </c>
+      <c r="E260" t="inlineStr">
+        <is>
+          <t>mladé listy</t>
+        </is>
+      </c>
+      <c r="F260" t="inlineStr">
+        <is>
+          <t>potrava</t>
+        </is>
+      </c>
+      <c r="G260" t="inlineStr">
+        <is>
+          <t>časné listy syrové / do polévky</t>
+        </is>
+      </c>
+      <c r="H260" t="inlineStr">
+        <is>
+          <t>téměř zapomenuté</t>
+        </is>
+      </c>
+      <c r="I260" t="inlineStr">
+        <is>
+          <t>střední</t>
+        </is>
+      </c>
+      <c r="J260" t="inlineStr">
+        <is>
+          <t>vlhčí listnaté lesy, stinné lemy, humózní svahy a starší parky</t>
+        </is>
+      </c>
+      <c r="K260" t="inlineStr">
+        <is>
+          <t>III–IV</t>
+        </is>
+      </c>
+      <c r="L260" t="inlineStr">
+        <is>
+          <t>měkké přízemní listy ještě před hrubnutím a před plným rozkvětem</t>
+        </is>
+      </c>
+      <c r="M260" t="inlineStr">
+        <is>
+          <t>Sbírat jen pár mladých listů z hojnějších trsů, použít je syrové do směsi nebo krátce přidat do jarní polévky.</t>
+        </is>
+      </c>
+      <c r="N260" t="inlineStr">
+        <is>
+          <t>Velmi raná a nenápadná lesní listová zelenina pro uživatele, kteří chtějí jít hlouběji než po běžných plevelech.</t>
+        </is>
+      </c>
+      <c r="O260" t="inlineStr">
+        <is>
+          <t>jemná, měkká, nevýrazně zelená</t>
+        </is>
+      </c>
+      <c r="P260" t="inlineStr">
+        <is>
+          <t>slabě listový</t>
+        </is>
+      </c>
+      <c r="Q260" t="inlineStr">
+        <is>
+          <t>neaplikovatelné</t>
+        </is>
+      </c>
+      <c r="R260" t="inlineStr">
+        <is>
+          <t>Sbírat jen tam, kde je druh opravdu hojný; nejde o rostlinu pro velkoobjemový sběr.</t>
+        </is>
+      </c>
+      <c r="S260" t="inlineStr"/>
+      <c r="T260" t="inlineStr">
+        <is>
+          <t>V lučních a chráněných lokalitách být zdrženlivý a sbírat jen malé množství z míst, kde je sběr legální.</t>
+        </is>
+      </c>
+      <c r="U260" t="inlineStr">
+        <is>
+          <t>kurátorovaný botanický zdroj</t>
+        </is>
+      </c>
+      <c r="V260" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="W260" t="inlineStr">
+        <is>
+          <t>S98</t>
+        </is>
+      </c>
+      <c r="X260" t="inlineStr"/>
+      <c r="Y260" t="inlineStr">
+        <is>
+          <t>Březnové rozšíření směrem k velmi časným listům stinných stanovišť.</t>
+        </is>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" t="inlineStr">
+        <is>
+          <t>R260</t>
+        </is>
+      </c>
+      <c r="B261" t="inlineStr">
+        <is>
+          <t>Primula veris</t>
+        </is>
+      </c>
+      <c r="C261" t="inlineStr">
+        <is>
+          <t>prvosenka jarní</t>
+        </is>
+      </c>
+      <c r="D261" t="inlineStr">
+        <is>
+          <t>původní, lokálně běžná</t>
+        </is>
+      </c>
+      <c r="E261" t="inlineStr">
+        <is>
+          <t>mladé listy</t>
+        </is>
+      </c>
+      <c r="F261" t="inlineStr">
+        <is>
+          <t>potrava</t>
+        </is>
+      </c>
+      <c r="G261" t="inlineStr">
+        <is>
+          <t>časné listy syrové / do polévky / jako čajová náhražka</t>
+        </is>
+      </c>
+      <c r="H261" t="inlineStr">
+        <is>
+          <t>téměř zapomenuté</t>
+        </is>
+      </c>
+      <c r="I261" t="inlineStr">
+        <is>
+          <t>střední</t>
+        </is>
+      </c>
+      <c r="J261" t="inlineStr">
+        <is>
+          <t>světlejší louky, remízky, okraje lesů, suché až mezofilní trávníky</t>
+        </is>
+      </c>
+      <c r="K261" t="inlineStr">
+        <is>
+          <t>III–IV</t>
+        </is>
+      </c>
+      <c r="L261" t="inlineStr">
+        <is>
+          <t>nejmladší listy v přízemní růžici před plným kvetením</t>
+        </is>
+      </c>
+      <c r="M261" t="inlineStr">
+        <is>
+          <t>Mladé listy přidávat v malém množství do směsí nebo do jarní polévky; lze je i sušit a používat jako jednoduchou čajovou náhražku.</t>
+        </is>
+      </c>
+      <c r="N261" t="inlineStr">
+        <is>
+          <t>Časná jarní listová surovina, která dává smysl hlavně pro rozšíření repertoáru o opravdu časné luční druhy.</t>
+        </is>
+      </c>
+      <c r="O261" t="inlineStr">
+        <is>
+          <t>spíše jemná, lehce bylinná</t>
+        </is>
+      </c>
+      <c r="P261" t="inlineStr">
+        <is>
+          <t>slabý zelený</t>
+        </is>
+      </c>
+      <c r="Q261" t="inlineStr">
+        <is>
+          <t>neaplikovatelné</t>
+        </is>
+      </c>
+      <c r="R261" t="inlineStr">
+        <is>
+          <t>Listy nejsou chuťově výjimečné, takže sběr má smysl jen střídmý; nepustošit květné louky kvůli hrsti listů.</t>
+        </is>
+      </c>
+      <c r="S261" t="inlineStr">
+        <is>
+          <t>U citlivých osob opatrnost na saponiny a při souběžném užívání léků na srážlivost.</t>
+        </is>
+      </c>
+      <c r="T261" t="inlineStr">
+        <is>
+          <t>Sbírat jen střídmě a tam, kde je druh na lokalitě hojný a sběr je legální.</t>
+        </is>
+      </c>
+      <c r="U261" t="inlineStr">
+        <is>
+          <t>kurátorovaný botanický zdroj</t>
+        </is>
+      </c>
+      <c r="V261" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="W261" t="inlineStr">
+        <is>
+          <t>S97</t>
+        </is>
+      </c>
+      <c r="X261" t="inlineStr"/>
+      <c r="Y261" t="inlineStr">
+        <is>
+          <t>Březnová vlna se rozšiřuje i o časně sbíratelné prvosenkové listy.</t>
+        </is>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" t="inlineStr">
+        <is>
+          <t>R261</t>
+        </is>
+      </c>
+      <c r="B262" t="inlineStr">
+        <is>
+          <t>Primula veris</t>
+        </is>
+      </c>
+      <c r="C262" t="inlineStr">
+        <is>
+          <t>prvosenka jarní</t>
+        </is>
+      </c>
+      <c r="D262" t="inlineStr">
+        <is>
+          <t>původní, lokálně běžná</t>
+        </is>
+      </c>
+      <c r="E262" t="inlineStr">
+        <is>
+          <t>květy</t>
+        </is>
+      </c>
+      <c r="F262" t="inlineStr">
+        <is>
+          <t>potrava</t>
+        </is>
+      </c>
+      <c r="G262" t="inlineStr">
+        <is>
+          <t>květy do salátu / ozdoby / konzervy</t>
+        </is>
+      </c>
+      <c r="H262" t="inlineStr">
+        <is>
+          <t>méně známé</t>
+        </is>
+      </c>
+      <c r="I262" t="inlineStr">
+        <is>
+          <t>střední</t>
+        </is>
+      </c>
+      <c r="J262" t="inlineStr">
+        <is>
+          <t>světlejší louky, remízky, okraje lesů, suché až mezofilní trávníky</t>
+        </is>
+      </c>
+      <c r="K262" t="inlineStr">
+        <is>
+          <t>IV–V</t>
+        </is>
+      </c>
+      <c r="L262" t="inlineStr">
+        <is>
+          <t>čerstvě rozvinuté voňavé květy</t>
+        </is>
+      </c>
+      <c r="M262" t="inlineStr">
+        <is>
+          <t>Květy používat čerstvé jako jedlou ozdobu nebo je zpracovat do menší domácí konzervy, případně do tradičněji laděného jarního květního nápoje.</t>
+        </is>
+      </c>
+      <c r="N262" t="inlineStr">
+        <is>
+          <t>Jemná květní jarní surovina s přesahem do domácích sladších konzerv a tradičnějších květních nápojů.</t>
+        </is>
+      </c>
+      <c r="O262" t="inlineStr">
+        <is>
+          <t>jemně květní, lehce medová</t>
+        </is>
+      </c>
+      <c r="P262" t="inlineStr">
+        <is>
+          <t>výrazněji jarně květní</t>
+        </is>
+      </c>
+      <c r="Q262" t="inlineStr">
+        <is>
+          <t>neaplikovatelné</t>
+        </is>
+      </c>
+      <c r="R262" t="inlineStr">
+        <is>
+          <t>Netrhat ve velkém celé květy z málo početných lokalit; sběr má být spíš symbolický než objemový.</t>
+        </is>
+      </c>
+      <c r="S262" t="inlineStr">
+        <is>
+          <t>U citlivých osob opatrnost na saponiny; při užívání antikoagulancií a v těhotenství konzervativní přístup.</t>
+        </is>
+      </c>
+      <c r="T262" t="inlineStr">
+        <is>
+          <t>Sbírat jen malé množství z hojných porostů a vyhnout se chráněným nebo citlivým lokalitám.</t>
+        </is>
+      </c>
+      <c r="U262" t="inlineStr">
+        <is>
+          <t>kurátorovaný botanický zdroj</t>
+        </is>
+      </c>
+      <c r="V262" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="W262" t="inlineStr">
+        <is>
+          <t>S97</t>
+        </is>
+      </c>
+      <c r="X262" t="inlineStr"/>
+      <c r="Y262" t="inlineStr">
+        <is>
+          <t>Přemosťuje březen do května a dává datasetu i jemnější jarní květní konzervové směry.</t>
+        </is>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" t="inlineStr">
+        <is>
+          <t>R262</t>
+        </is>
+      </c>
+      <c r="B263" t="inlineStr">
+        <is>
+          <t>Lamium purpureum</t>
+        </is>
+      </c>
+      <c r="C263" t="inlineStr">
+        <is>
+          <t>hluchavka nachová</t>
+        </is>
+      </c>
+      <c r="D263" t="inlineStr">
+        <is>
+          <t>původní, velmi běžná</t>
+        </is>
+      </c>
+      <c r="E263" t="inlineStr">
+        <is>
+          <t>mladé listy a vrcholky</t>
+        </is>
+      </c>
+      <c r="F263" t="inlineStr">
+        <is>
+          <t>potrava</t>
+        </is>
+      </c>
+      <c r="G263" t="inlineStr">
+        <is>
+          <t>mladé vrcholky syrové / krátce vařené</t>
+        </is>
+      </c>
+      <c r="H263" t="inlineStr">
+        <is>
+          <t>méně známé</t>
+        </is>
+      </c>
+      <c r="I263" t="inlineStr">
+        <is>
+          <t>vysoká</t>
+        </is>
+      </c>
+      <c r="J263" t="inlineStr">
+        <is>
+          <t>zahrady, záhony, okraje cest, pole, ruderální místa, spáry a městské kouty</t>
+        </is>
+      </c>
+      <c r="K263" t="inlineStr">
+        <is>
+          <t>III–V</t>
+        </is>
+      </c>
+      <c r="L263" t="inlineStr">
+        <is>
+          <t>měkké vrcholky před zhrubnutím a před plným odkvětem</t>
+        </is>
+      </c>
+      <c r="M263" t="inlineStr">
+        <is>
+          <t>Vrcholky používat syrové po menším množství do jarních směsí nebo je krátce podusit s další zelení jako městsky dostupnou listovou složku.</t>
+        </is>
+      </c>
+      <c r="N263" t="inlineStr">
+        <is>
+          <t>Nenápadná a snadno dostupná jarní zeleň z mikrostanovišť, která lidé obvykle míjejí bez povšimnutí.</t>
+        </is>
+      </c>
+      <c r="O263" t="inlineStr">
+        <is>
+          <t>jemná, lehce zelená, mírně zemitá</t>
+        </is>
+      </c>
+      <c r="P263" t="inlineStr">
+        <is>
+          <t>slabě bylinný</t>
+        </is>
+      </c>
+      <c r="Q263" t="inlineStr">
+        <is>
+          <t>neaplikovatelné</t>
+        </is>
+      </c>
+      <c r="R263" t="inlineStr">
+        <is>
+          <t>Sbírat jen z opravdu čistých míst mimo psí zóny, krajnice a chemicky ošetřené záhony.</t>
+        </is>
+      </c>
+      <c r="S263" t="inlineStr"/>
+      <c r="T263" t="inlineStr">
+        <is>
+          <t>Velmi běžný druh; prakticky nejbezpečnější je sběr ze zahrad nebo čistých městských mikrostanovišť.</t>
+        </is>
+      </c>
+      <c r="U263" t="inlineStr">
+        <is>
+          <t>kurátorovaný botanický zdroj</t>
+        </is>
+      </c>
+      <c r="V263" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="W263" t="inlineStr">
+        <is>
+          <t>S99</t>
+        </is>
+      </c>
+      <c r="X263" t="inlineStr"/>
+      <c r="Y263" t="inlineStr">
+        <is>
+          <t>Březnově-dubnová vlna přidává i málo zmiňované, ale velmi dostupné městské a zahradní druhy.</t>
+        </is>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" t="inlineStr">
+        <is>
+          <t>R263</t>
+        </is>
+      </c>
+      <c r="B264" t="inlineStr">
+        <is>
+          <t>Lamium album</t>
+        </is>
+      </c>
+      <c r="C264" t="inlineStr">
+        <is>
+          <t>hluchavka bílá</t>
+        </is>
+      </c>
+      <c r="D264" t="inlineStr">
+        <is>
+          <t>původní, běžná</t>
+        </is>
+      </c>
+      <c r="E264" t="inlineStr">
+        <is>
+          <t>mladé listy</t>
+        </is>
+      </c>
+      <c r="F264" t="inlineStr">
+        <is>
+          <t>potrava</t>
+        </is>
+      </c>
+      <c r="G264" t="inlineStr">
+        <is>
+          <t>mladé listy syrové / vařené</t>
+        </is>
+      </c>
+      <c r="H264" t="inlineStr">
+        <is>
+          <t>méně známé</t>
+        </is>
+      </c>
+      <c r="I264" t="inlineStr">
+        <is>
+          <t>střední až vysoká</t>
+        </is>
+      </c>
+      <c r="J264" t="inlineStr">
+        <is>
+          <t>živé ploty, okraje cest, křoviny, lesní lemy, zahrady, ruderální místa</t>
+        </is>
+      </c>
+      <c r="K264" t="inlineStr">
+        <is>
+          <t>III–V</t>
+        </is>
+      </c>
+      <c r="L264" t="inlineStr">
+        <is>
+          <t>nejmladší listy a měkké vrcholky před zhrubnutím</t>
+        </is>
+      </c>
+      <c r="M264" t="inlineStr">
+        <is>
+          <t>Mladé listy použít syrové do směsí nebo je vařit spolu s další jarní zelení; samostatně jsou spíš jemné než výrazné.</t>
+        </is>
+      </c>
+      <c r="N264" t="inlineStr">
+        <is>
+          <t>Další tichý, ale použitelný jarní druh z živých plotů a lemů, vhodný hlavně do směsných sběrů.</t>
+        </is>
+      </c>
+      <c r="O264" t="inlineStr">
+        <is>
+          <t>jemná, lehce travnatá</t>
+        </is>
+      </c>
+      <c r="P264" t="inlineStr">
+        <is>
+          <t>slabě bylinný</t>
+        </is>
+      </c>
+      <c r="Q264" t="inlineStr">
+        <is>
+          <t>neaplikovatelné</t>
+        </is>
+      </c>
+      <c r="R264" t="inlineStr">
+        <is>
+          <t>Sbírat z čistých míst a nesahat po listech z okrasných nebo chemicky ošetřených výsadeb.</t>
+        </is>
+      </c>
+      <c r="S264" t="inlineStr"/>
+      <c r="T264" t="inlineStr">
+        <is>
+          <t>Sbírat střídmě a hlavně z běžných, snadno přístupných a čistých porostů.</t>
+        </is>
+      </c>
+      <c r="U264" t="inlineStr">
+        <is>
+          <t>kurátorovaný botanický zdroj</t>
+        </is>
+      </c>
+      <c r="V264" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="W264" t="inlineStr">
+        <is>
+          <t>S100</t>
+        </is>
+      </c>
+      <c r="X264" t="inlineStr"/>
+      <c r="Y264" t="inlineStr">
+        <is>
+          <t>Posiluje březnový a dubnový repertoár o další málo doceňovanou hluchavku.</t>
+        </is>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" t="inlineStr">
+        <is>
+          <t>R264</t>
+        </is>
+      </c>
+      <c r="B265" t="inlineStr">
+        <is>
+          <t>Lamium album</t>
+        </is>
+      </c>
+      <c r="C265" t="inlineStr">
+        <is>
+          <t>hluchavka bílá</t>
+        </is>
+      </c>
+      <c r="D265" t="inlineStr">
+        <is>
+          <t>původní, běžná</t>
+        </is>
+      </c>
+      <c r="E265" t="inlineStr">
+        <is>
+          <t>květy</t>
+        </is>
+      </c>
+      <c r="F265" t="inlineStr">
+        <is>
+          <t>pití</t>
+        </is>
+      </c>
+      <c r="G265" t="inlineStr">
+        <is>
+          <t>sušené květy na jemný čaj</t>
+        </is>
+      </c>
+      <c r="H265" t="inlineStr">
+        <is>
+          <t>téměř zapomenuté</t>
+        </is>
+      </c>
+      <c r="I265" t="inlineStr">
+        <is>
+          <t>střední</t>
+        </is>
+      </c>
+      <c r="J265" t="inlineStr">
+        <is>
+          <t>živé ploty, křoviny, lemy cest, zahrady a ruderální okraje</t>
+        </is>
+      </c>
+      <c r="K265" t="inlineStr">
+        <is>
+          <t>V–IX + sušení</t>
+        </is>
+      </c>
+      <c r="L265" t="inlineStr">
+        <is>
+          <t>čerstvě rozvité bílé květy sbírané za sucha</t>
+        </is>
+      </c>
+      <c r="M265" t="inlineStr">
+        <is>
+          <t>Květy šetrně usušit a používat na jemný bylinný čaj nebo jako zjemňující složku domácích směsí.</t>
+        </is>
+      </c>
+      <c r="N265" t="inlineStr">
+        <is>
+          <t>Lehká a poměrně příjemná květní čajovina z velmi běžné, ale přehlížené rostliny.</t>
+        </is>
+      </c>
+      <c r="O265" t="inlineStr">
+        <is>
+          <t>jemná, lehce nasládlá, květní</t>
+        </is>
+      </c>
+      <c r="P265" t="inlineStr">
+        <is>
+          <t>slabě medový</t>
+        </is>
+      </c>
+      <c r="Q265" t="inlineStr">
+        <is>
+          <t>neaplikovatelné</t>
+        </is>
+      </c>
+      <c r="R265" t="inlineStr">
+        <is>
+          <t>Sbírat jen suché, čisté květy; nezapařit je při sušení a brát je spíš jako jemnou čajovou surovinu než jako silnou bylinu.</t>
+        </is>
+      </c>
+      <c r="S265" t="inlineStr"/>
+      <c r="T265" t="inlineStr">
+        <is>
+          <t>Běžný druh; vhodný hlavně ze zahradních a křovinných porostů bez chemického ošetření.</t>
+        </is>
+      </c>
+      <c r="U265" t="inlineStr">
+        <is>
+          <t>kurátorovaný botanický zdroj</t>
+        </is>
+      </c>
+      <c r="V265" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="W265" t="inlineStr">
+        <is>
+          <t>S100</t>
+        </is>
+      </c>
+      <c r="X265" t="inlineStr"/>
+      <c r="Y265" t="inlineStr">
+        <is>
+          <t>Květnová vlna vědomě přidává i tiché čajové suroviny, které nejsou v moderním foragingu moc vidět.</t>
+        </is>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" t="inlineStr">
+        <is>
+          <t>R265</t>
+        </is>
+      </c>
+      <c r="B266" t="inlineStr">
+        <is>
+          <t>Alliaria petiolata</t>
+        </is>
+      </c>
+      <c r="C266" t="inlineStr">
+        <is>
+          <t>česnáček lékařský</t>
+        </is>
+      </c>
+      <c r="D266" t="inlineStr">
+        <is>
+          <t>původní, běžný</t>
+        </is>
+      </c>
+      <c r="E266" t="inlineStr">
+        <is>
+          <t>mladé listy</t>
+        </is>
+      </c>
+      <c r="F266" t="inlineStr">
+        <is>
+          <t>potrava</t>
+        </is>
+      </c>
+      <c r="G266" t="inlineStr">
+        <is>
+          <t>časné listy do salátu / jako dochucení</t>
+        </is>
+      </c>
+      <c r="H266" t="inlineStr">
+        <is>
+          <t>méně známé</t>
+        </is>
+      </c>
+      <c r="I266" t="inlineStr">
+        <is>
+          <t>vysoká</t>
+        </is>
+      </c>
+      <c r="J266" t="inlineStr">
+        <is>
+          <t>křoviny, lesní lemy, stinnější zídky, staré sady, vlhčí polostinná místa</t>
+        </is>
+      </c>
+      <c r="K266" t="inlineStr">
+        <is>
+          <t>III–V</t>
+        </is>
+      </c>
+      <c r="L266" t="inlineStr">
+        <is>
+          <t>mladé listy před plným kvetením</t>
+        </is>
+      </c>
+      <c r="M266" t="inlineStr">
+        <is>
+          <t>Listy používat syrové do salátů a pomazánek nebo po malém množství do vařených jídel jako česnekově-hořčičné dochucení.</t>
+        </is>
+      </c>
+      <c r="N266" t="inlineStr">
+        <is>
+          <t>Brzy dostupná kořenná listová bylina, která dobře překlene období před česnekem medvědím a dalšími výraznějšími zeleněmi.</t>
+        </is>
+      </c>
+      <c r="O266" t="inlineStr">
+        <is>
+          <t>česnekově-hořčičná, lehce štiplavá</t>
+        </is>
+      </c>
+      <c r="P266" t="inlineStr">
+        <is>
+          <t>česnekový, brukvovitý</t>
+        </is>
+      </c>
+      <c r="Q266" t="inlineStr">
+        <is>
+          <t>neaplikovatelné</t>
+        </is>
+      </c>
+      <c r="R266" t="inlineStr">
+        <is>
+          <t>Jako brukvovitá může ve větším množství dráždit citlivější trávení; sbírat mimo znečištěná městská stinná místa.</t>
+        </is>
+      </c>
+      <c r="S266" t="inlineStr">
+        <is>
+          <t>U citlivějších osob opatrnost při vyšším množství brukvovitých.</t>
+        </is>
+      </c>
+      <c r="T266" t="inlineStr">
+        <is>
+          <t>Běžný druh; sběr v malém z běžných porostů je prakticky dostupný, ale vždy mimo chráněné lokality a znečištěná místa.</t>
+        </is>
+      </c>
+      <c r="U266" t="inlineStr">
+        <is>
+          <t>kurátorovaný botanický zdroj</t>
+        </is>
+      </c>
+      <c r="V266" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="W266" t="inlineStr">
+        <is>
+          <t>S101</t>
+        </is>
+      </c>
+      <c r="X266" t="inlineStr"/>
+      <c r="Y266" t="inlineStr">
+        <is>
+          <t>Přidává do března a dubna silnější chuťový most mezi listovou zelení a kořením.</t>
+        </is>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" t="inlineStr">
+        <is>
+          <t>R266</t>
+        </is>
+      </c>
+      <c r="B267" t="inlineStr">
+        <is>
+          <t>Alliaria petiolata</t>
+        </is>
+      </c>
+      <c r="C267" t="inlineStr">
+        <is>
+          <t>česnáček lékařský</t>
+        </is>
+      </c>
+      <c r="D267" t="inlineStr">
+        <is>
+          <t>původní, běžný</t>
+        </is>
+      </c>
+      <c r="E267" t="inlineStr">
+        <is>
+          <t>květy a mladé šešulky</t>
+        </is>
+      </c>
+      <c r="F267" t="inlineStr">
+        <is>
+          <t>potrava</t>
+        </is>
+      </c>
+      <c r="G267" t="inlineStr">
+        <is>
+          <t>květy a mladé šešulky syrové jako kořeněná složka</t>
+        </is>
+      </c>
+      <c r="H267" t="inlineStr">
+        <is>
+          <t>téměř zapomenuté</t>
+        </is>
+      </c>
+      <c r="I267" t="inlineStr">
+        <is>
+          <t>střední až vysoká</t>
+        </is>
+      </c>
+      <c r="J267" t="inlineStr">
+        <is>
+          <t>křoviny, lesní lemy, starší parky, zídky a stinná rumiště</t>
+        </is>
+      </c>
+      <c r="K267" t="inlineStr">
+        <is>
+          <t>V–VI</t>
+        </is>
+      </c>
+      <c r="L267" t="inlineStr">
+        <is>
+          <t>otevřené květy a velmi mladé měkké šešulky</t>
+        </is>
+      </c>
+      <c r="M267" t="inlineStr">
+        <is>
+          <t>Květy a ještě měkké mladé šešulky používat syrové po malém množství jako pikantní, česnekově-hořčičný detail do jídel.</t>
+        </is>
+      </c>
+      <c r="N267" t="inlineStr">
+        <is>
+          <t>Květnová nadstavba česnáčku, která rozšiřuje sběr i po odeznění nejlepších listů.</t>
+        </is>
+      </c>
+      <c r="O267" t="inlineStr">
+        <is>
+          <t>pikantní, česnekově-hořčičný</t>
+        </is>
+      </c>
+      <c r="P267" t="inlineStr">
+        <is>
+          <t>výrazně brukvovitý</t>
+        </is>
+      </c>
+      <c r="Q267" t="inlineStr">
+        <is>
+          <t>neaplikovatelné</t>
+        </is>
+      </c>
+      <c r="R267" t="inlineStr">
+        <is>
+          <t>Sbírat jen mladé, měkké šešulky; starší části rychle hrubnou a chuť bývá tvrdší.</t>
+        </is>
+      </c>
+      <c r="S267" t="inlineStr">
+        <is>
+          <t>U citlivějších osob opatrnost při vyšším množství brukvovitých.</t>
+        </is>
+      </c>
+      <c r="T267" t="inlineStr">
+        <is>
+          <t>Běžný druh; sbírat střídmě a jen z čistých míst.</t>
+        </is>
+      </c>
+      <c r="U267" t="inlineStr">
+        <is>
+          <t>kurátorovaný botanický zdroj</t>
+        </is>
+      </c>
+      <c r="V267" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="W267" t="inlineStr">
+        <is>
+          <t>S101</t>
+        </is>
+      </c>
+      <c r="X267" t="inlineStr"/>
+      <c r="Y267" t="inlineStr">
+        <is>
+          <t>Květnová vlna doplňuje i méně zmiňované pozdější části česnáčku.</t>
+        </is>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" t="inlineStr">
+        <is>
+          <t>R267</t>
+        </is>
+      </c>
+      <c r="B268" t="inlineStr">
+        <is>
+          <t>Robinia pseudoacacia</t>
+        </is>
+      </c>
+      <c r="C268" t="inlineStr">
+        <is>
+          <t>trnovník akát</t>
+        </is>
+      </c>
+      <c r="D268" t="inlineStr">
+        <is>
+          <t>nepůvodní, zdomácnělý a běžný</t>
+        </is>
+      </c>
+      <c r="E268" t="inlineStr">
+        <is>
+          <t>květy</t>
+        </is>
+      </c>
+      <c r="F268" t="inlineStr">
+        <is>
+          <t>potrava</t>
+        </is>
+      </c>
+      <c r="G268" t="inlineStr">
+        <is>
+          <t>květy vařené / nápoj / zavařenina</t>
+        </is>
+      </c>
+      <c r="H268" t="inlineStr">
+        <is>
+          <t>méně známé</t>
+        </is>
+      </c>
+      <c r="I268" t="inlineStr">
+        <is>
+          <t>střední</t>
+        </is>
+      </c>
+      <c r="J268" t="inlineStr">
+        <is>
+          <t>teplejší stráně, aleje, remízky, suché meze, městské a příměstské výsadby</t>
+        </is>
+      </c>
+      <c r="K268" t="inlineStr">
+        <is>
+          <t>V–VI</t>
+        </is>
+      </c>
+      <c r="L268" t="inlineStr">
+        <is>
+          <t>čerstvě rozvinuté voňavé květní hrozny</t>
+        </is>
+      </c>
+      <c r="M268" t="inlineStr">
+        <is>
+          <t>Sbírat jen samotné květy bez zelených částí a používat je vařené do sladších jídel, do domácí zavařeniny nebo na voňavý květní nápoj.</t>
+        </is>
+      </c>
+      <c r="N268" t="inlineStr">
+        <is>
+          <t>Výrazně aromatická květnová surovina s potenciálem pro nápojové a sladké uchování.</t>
+        </is>
+      </c>
+      <c r="O268" t="inlineStr">
+        <is>
+          <t>sladce květní, lehce vanilkový</t>
+        </is>
+      </c>
+      <c r="P268" t="inlineStr">
+        <is>
+          <t>silně medově květní</t>
+        </is>
+      </c>
+      <c r="Q268" t="inlineStr">
+        <is>
+          <t>neaplikovatelné</t>
+        </is>
+      </c>
+      <c r="R268" t="inlineStr">
+        <is>
+          <t>Jedlé jsou jen květy; listy, kůra, semena a další části jsou toxické. Nesbírat z prašných ulic ani stromů po chemickém zásahu.</t>
+        </is>
+      </c>
+      <c r="S268" t="inlineStr">
+        <is>
+          <t>Používat jen květy a při první práci s druhem začít opatrně malým množstvím.</t>
+        </is>
+      </c>
+      <c r="T268" t="inlineStr">
+        <is>
+          <t>Běžný zdomácnělý druh; sběr jen z čistých míst a bez poškozování výhonů či stromů.</t>
+        </is>
+      </c>
+      <c r="U268" t="inlineStr">
+        <is>
+          <t>kurátorovaný botanický zdroj</t>
+        </is>
+      </c>
+      <c r="V268" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="W268" t="inlineStr">
+        <is>
+          <t>S102</t>
+        </is>
+      </c>
+      <c r="X268" t="inlineStr"/>
+      <c r="Y268" t="inlineStr">
+        <is>
+          <t>Květnová vlna přidává i silně voňavé květní využití s velkým důrazem na to, že jedlé jsou opravdu jen květy.</t>
+        </is>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" t="inlineStr">
+        <is>
+          <t>R268</t>
+        </is>
+      </c>
+      <c r="B269" t="inlineStr">
+        <is>
+          <t>Humulus lupulus</t>
+        </is>
+      </c>
+      <c r="C269" t="inlineStr">
+        <is>
+          <t>chmel otáčivý</t>
+        </is>
+      </c>
+      <c r="D269" t="inlineStr">
+        <is>
+          <t>původní, běžný</t>
+        </is>
+      </c>
+      <c r="E269" t="inlineStr">
+        <is>
+          <t>mladé výhonky a listy</t>
+        </is>
+      </c>
+      <c r="F269" t="inlineStr">
+        <is>
+          <t>potrava</t>
+        </is>
+      </c>
+      <c r="G269" t="inlineStr">
+        <is>
+          <t>jarní výhonky a listy vařené / syrové po menším množství</t>
+        </is>
+      </c>
+      <c r="H269" t="inlineStr">
+        <is>
+          <t>téměř zapomenuté</t>
+        </is>
+      </c>
+      <c r="I269" t="inlineStr">
+        <is>
+          <t>střední</t>
+        </is>
+      </c>
+      <c r="J269" t="inlineStr">
+        <is>
+          <t>křoviny, břehy, nivy, remízky, okraje lesů a staré ploty</t>
+        </is>
+      </c>
+      <c r="K269" t="inlineStr">
+        <is>
+          <t>IV–V</t>
+        </is>
+      </c>
+      <c r="L269" t="inlineStr">
+        <is>
+          <t>nejmladší špičky výhonů a měkké listy před koncem května</t>
+        </is>
+      </c>
+      <c r="M269" t="inlineStr">
+        <is>
+          <t>Mladé výhonky krátce vařit nebo podusit jako jarní zeleninu; nejmladší listy lze po malém množství přidat i syrové do směsí.</t>
+        </is>
+      </c>
+      <c r="N269" t="inlineStr">
+        <is>
+          <t>Krátké a hodnotné květnové okno pro výraznější divoké výhonky, které většina lidí spojuje spíš s pivem než s jídlem.</t>
+        </is>
+      </c>
+      <c r="O269" t="inlineStr">
+        <is>
+          <t>zelený, lehce chmelový, specifický</t>
+        </is>
+      </c>
+      <c r="P269" t="inlineStr">
+        <is>
+          <t>pryskyřičně bylinný</t>
+        </is>
+      </c>
+      <c r="Q269" t="inlineStr">
+        <is>
+          <t>neaplikovatelné</t>
+        </is>
+      </c>
+      <c r="R269" t="inlineStr">
+        <is>
+          <t>Používat jen opravdu mladé části před koncem května; starší rychle hrubnou a ztrácejí kuchyňskou hodnotu.</t>
+        </is>
+      </c>
+      <c r="S269" t="inlineStr"/>
+      <c r="T269" t="inlineStr">
+        <is>
+          <t>Sbírat jednotlivé špičky z hojných porostů bez strhávání celých lian.</t>
+        </is>
+      </c>
+      <c r="U269" t="inlineStr">
+        <is>
+          <t>kurátorovaný botanický zdroj</t>
+        </is>
+      </c>
+      <c r="V269" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="W269" t="inlineStr">
+        <is>
+          <t>S103</t>
+        </is>
+      </c>
+      <c r="X269" t="inlineStr"/>
+      <c r="Y269" t="inlineStr">
+        <is>
+          <t>Květnová vlna rozšiřuje výhonkový sběr i na druhy, které jsou dnes v kuchyňském použití skoro neviditelné.</t>
+        </is>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" t="inlineStr">
+        <is>
+          <t>R269</t>
+        </is>
+      </c>
+      <c r="B270" t="inlineStr">
+        <is>
+          <t>Epilobium angustifolium</t>
+        </is>
+      </c>
+      <c r="C270" t="inlineStr">
+        <is>
+          <t>vrbovka úzkolistá</t>
+        </is>
+      </c>
+      <c r="D270" t="inlineStr">
+        <is>
+          <t>původní, běžná</t>
+        </is>
+      </c>
+      <c r="E270" t="inlineStr">
+        <is>
+          <t>mladé výhonky, listy a poupata</t>
+        </is>
+      </c>
+      <c r="F270" t="inlineStr">
+        <is>
+          <t>potrava</t>
+        </is>
+      </c>
+      <c r="G270" t="inlineStr">
+        <is>
+          <t>jarní výhonky syrové / vařené / ledničkové pickles</t>
+        </is>
+      </c>
+      <c r="H270" t="inlineStr">
+        <is>
+          <t>téměř zapomenuté</t>
+        </is>
+      </c>
+      <c r="I270" t="inlineStr">
+        <is>
+          <t>střední</t>
+        </is>
+      </c>
+      <c r="J270" t="inlineStr">
+        <is>
+          <t>lesní paseky, okraje cest v horách a podhůří, světliny, náspy, disturbované lesní okraje</t>
+        </is>
+      </c>
+      <c r="K270" t="inlineStr">
+        <is>
+          <t>V–VI</t>
+        </is>
+      </c>
+      <c r="L270" t="inlineStr">
+        <is>
+          <t>mladé šťavnaté výhonky, jemné listy a neotevřená poupata před plným květem</t>
+        </is>
+      </c>
+      <c r="M270" t="inlineStr">
+        <is>
+          <t>Mladé výhonky a poupata používat syrové po menším množství, krátce je napařit nebo je naložit do ledničkových pickles.</t>
+        </is>
+      </c>
+      <c r="N270" t="inlineStr">
+        <is>
+          <t>Květnová a raně letní výhonková zelenina s překvapivě širokým rozsahem od čerstvého použití po jemnější pickles.</t>
+        </is>
+      </c>
+      <c r="O270" t="inlineStr">
+        <is>
+          <t>jemně zelený, někdy lehce peprný</t>
+        </is>
+      </c>
+      <c r="P270" t="inlineStr">
+        <is>
+          <t>čerstvě bylinný</t>
+        </is>
+      </c>
+      <c r="Q270" t="inlineStr">
+        <is>
+          <t>neaplikovatelné</t>
+        </is>
+      </c>
+      <c r="R270" t="inlineStr">
+        <is>
+          <t>Pozdější listy a stonky rychle tuhnou a hořknou; sběr má smysl jen opravdu časný a z čistých lokalit.</t>
+        </is>
+      </c>
+      <c r="S270" t="inlineStr"/>
+      <c r="T270" t="inlineStr">
+        <is>
+          <t>Sbírat střídmě jen vrcholové části z běžných porostů a neničit celé plochy mladých výhonů.</t>
+        </is>
+      </c>
+      <c r="U270" t="inlineStr">
+        <is>
+          <t>kurátorovaný botanický + extension zdroj</t>
+        </is>
+      </c>
+      <c r="V270" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="W270" t="inlineStr">
+        <is>
+          <t>S104</t>
+        </is>
+      </c>
+      <c r="X270" t="inlineStr">
+        <is>
+          <t>S105</t>
+        </is>
+      </c>
+      <c r="Y270" t="inlineStr">
+        <is>
+          <t>Květnová vlna přidává i rostlinu, která umí spojit čerstvý sběr s praktickým uchováním.</t>
+        </is>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" t="inlineStr">
+        <is>
+          <t>R270</t>
+        </is>
+      </c>
+      <c r="B271" t="inlineStr">
+        <is>
+          <t>Epilobium angustifolium</t>
+        </is>
+      </c>
+      <c r="C271" t="inlineStr">
+        <is>
+          <t>vrbovka úzkolistá</t>
+        </is>
+      </c>
+      <c r="D271" t="inlineStr">
+        <is>
+          <t>původní, běžná</t>
+        </is>
+      </c>
+      <c r="E271" t="inlineStr">
+        <is>
+          <t>mladé listy a vrcholky</t>
+        </is>
+      </c>
+      <c r="F271" t="inlineStr">
+        <is>
+          <t>pití</t>
+        </is>
+      </c>
+      <c r="G271" t="inlineStr">
+        <is>
+          <t>fermentované a sušené listy na Ivan čaj</t>
+        </is>
+      </c>
+      <c r="H271" t="inlineStr">
+        <is>
+          <t>známé hlavně v zahraničí</t>
+        </is>
+      </c>
+      <c r="I271" t="inlineStr">
+        <is>
+          <t>střední</t>
+        </is>
+      </c>
+      <c r="J271" t="inlineStr">
+        <is>
+          <t>světliny, paseky, náspy, horské a podhorské disturbované lokality</t>
+        </is>
+      </c>
+      <c r="K271" t="inlineStr">
+        <is>
+          <t>V–VIII + fermentace + sušení</t>
+        </is>
+      </c>
+      <c r="L271" t="inlineStr">
+        <is>
+          <t>mladé listy a vrcholky v době před květem až na začátku nasazování poupat</t>
+        </is>
+      </c>
+      <c r="M271" t="inlineStr">
+        <is>
+          <t>Listy nebo měkké vrcholky nechat zavadnout, narušit pletiva, krátce fermentovat a následně dosušit jako nečerný bylinný 'Ivan čaj'.</t>
+        </is>
+      </c>
+      <c r="N271" t="inlineStr">
+        <is>
+          <t>Tradičněji laděná fermentovaná čajová surovina, známější na severu a východě Evropy než u nás.</t>
+        </is>
+      </c>
+      <c r="O271" t="inlineStr">
+        <is>
+          <t>hladký, tmavší bylinný, lehce ovocný</t>
+        </is>
+      </c>
+      <c r="P271" t="inlineStr">
+        <is>
+          <t>jemně fermentovaný, čajový</t>
+        </is>
+      </c>
+      <c r="Q271" t="inlineStr">
+        <is>
+          <t>neaplikovatelné</t>
+        </is>
+      </c>
+      <c r="R271" t="inlineStr">
+        <is>
+          <t>Bez správného zavadnutí, fermentace a dosušení může surovina plesnivět; sbírat jen zdravé listy bez prachu.</t>
+        </is>
+      </c>
+      <c r="S271" t="inlineStr">
+        <is>
+          <t>Jako u silnějších bylinných čajů začínat rozumným množstvím.</t>
+        </is>
+      </c>
+      <c r="T271" t="inlineStr">
+        <is>
+          <t>Sbírat jen z hojných porostů a neodřezávat celé plochy vrcholových částí.</t>
+        </is>
+      </c>
+      <c r="U271" t="inlineStr">
+        <is>
+          <t>kurátorovaný botanický + technologický zdroj</t>
+        </is>
+      </c>
+      <c r="V271" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="W271" t="inlineStr">
+        <is>
+          <t>S104</t>
+        </is>
+      </c>
+      <c r="X271" t="inlineStr">
+        <is>
+          <t>S106</t>
+        </is>
+      </c>
+      <c r="Y271" t="inlineStr">
+        <is>
+          <t>Květnové rozšíření vědomě přidává i zahraničněji známý fermentační směr, který odpovídá požadavku pronikat do tajů.</t>
+        </is>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" t="inlineStr">
+        <is>
+          <t>R271</t>
+        </is>
+      </c>
+      <c r="B272" t="inlineStr">
+        <is>
+          <t>Silene vulgaris</t>
+        </is>
+      </c>
+      <c r="C272" t="inlineStr">
+        <is>
+          <t>silenka nadmutá</t>
+        </is>
+      </c>
+      <c r="D272" t="inlineStr">
+        <is>
+          <t>původní, běžná lokálně</t>
+        </is>
+      </c>
+      <c r="E272" t="inlineStr">
+        <is>
+          <t>mladé výhonky a listy</t>
+        </is>
+      </c>
+      <c r="F272" t="inlineStr">
+        <is>
+          <t>potrava</t>
+        </is>
+      </c>
+      <c r="G272" t="inlineStr">
+        <is>
+          <t>mladé výhonky syrové / vařené před kvetením</t>
+        </is>
+      </c>
+      <c r="H272" t="inlineStr">
+        <is>
+          <t>známé hlavně v zahraničí</t>
+        </is>
+      </c>
+      <c r="I272" t="inlineStr">
+        <is>
+          <t>střední</t>
+        </is>
+      </c>
+      <c r="J272" t="inlineStr">
+        <is>
+          <t>suché meze, stráně, louky, okraje cest a kamenitější trávníky</t>
+        </is>
+      </c>
+      <c r="K272" t="inlineStr">
+        <is>
+          <t>V–VI</t>
+        </is>
+      </c>
+      <c r="L272" t="inlineStr">
+        <is>
+          <t>krátké mladé výhonky a listy před rozkvětem</t>
+        </is>
+      </c>
+      <c r="M272" t="inlineStr">
+        <is>
+          <t>Mladé výhonky jíst po menším množství syrové nebo je krátce povařit; při větší hořkosti je vhodné je předem blanšírovat.</t>
+        </is>
+      </c>
+      <c r="N272" t="inlineStr">
+        <is>
+          <t>Velmi ne-mainstreamová evropská jarní zelenina, která je u nás skoro neviditelná, ale jinde je ceněná.</t>
+        </is>
+      </c>
+      <c r="O272" t="inlineStr">
+        <is>
+          <t>sladce zelený s lehkou hořčinou</t>
+        </is>
+      </c>
+      <c r="P272" t="inlineStr">
+        <is>
+          <t>slabě bylinno-zelený</t>
+        </is>
+      </c>
+      <c r="Q272" t="inlineStr">
+        <is>
+          <t>neaplikovatelné</t>
+        </is>
+      </c>
+      <c r="R272" t="inlineStr">
+        <is>
+          <t>Používat jen mladé části před květem a ne ve velkých objemech kvůli obsahu saponinů.</t>
+        </is>
+      </c>
+      <c r="S272" t="inlineStr">
+        <is>
+          <t>Nevhodné ve velkých dávkách; při citlivém trávení začínat malým množstvím a preferovat tepelnou úpravu.</t>
+        </is>
+      </c>
+      <c r="T272" t="inlineStr">
+        <is>
+          <t>Sbírat střídmě jen z hojných porostů a ne z lokalit podezřelých na těžké kovy či jinou zátěž.</t>
+        </is>
+      </c>
+      <c r="U272" t="inlineStr">
+        <is>
+          <t>kurátorovaný botanický zdroj</t>
+        </is>
+      </c>
+      <c r="V272" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="W272" t="inlineStr">
+        <is>
+          <t>S107</t>
+        </is>
+      </c>
+      <c r="X272" t="inlineStr"/>
+      <c r="Y272" t="inlineStr">
+        <is>
+          <t>Květnová vlna úmyslně otevírá i druhy známé spíš v zahraničních regionálních kuchyních.</t>
+        </is>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" t="inlineStr">
+        <is>
+          <t>R272</t>
+        </is>
+      </c>
+      <c r="B273" t="inlineStr">
+        <is>
+          <t>Tragopogon pratensis</t>
+        </is>
+      </c>
+      <c r="C273" t="inlineStr">
+        <is>
+          <t>kozí brada luční</t>
+        </is>
+      </c>
+      <c r="D273" t="inlineStr">
+        <is>
+          <t>původní, běžná</t>
+        </is>
+      </c>
+      <c r="E273" t="inlineStr">
+        <is>
+          <t>mladé stonky, poupata a listy</t>
+        </is>
+      </c>
+      <c r="F273" t="inlineStr">
+        <is>
+          <t>potrava</t>
+        </is>
+      </c>
+      <c r="G273" t="inlineStr">
+        <is>
+          <t>květní stonky a poupata vařené jako 'divoký chřest'</t>
+        </is>
+      </c>
+      <c r="H273" t="inlineStr">
+        <is>
+          <t>téměř zapomenuté</t>
+        </is>
+      </c>
+      <c r="I273" t="inlineStr">
+        <is>
+          <t>střední</t>
+        </is>
+      </c>
+      <c r="J273" t="inlineStr">
+        <is>
+          <t>louky, meze, pastviny, náspy a světlejší ruderální okraje</t>
+        </is>
+      </c>
+      <c r="K273" t="inlineStr">
+        <is>
+          <t>V–VI</t>
+        </is>
+      </c>
+      <c r="L273" t="inlineStr">
+        <is>
+          <t>mladé květní stonky a poupata před otevřením květů</t>
+        </is>
+      </c>
+      <c r="M273" t="inlineStr">
+        <is>
+          <t>Květní stonky s poupaty krátce povařit nebo podusit a podávat podobně jako divoký chřest; listy a mladé výhonky lze přidat i do polévky.</t>
+        </is>
+      </c>
+      <c r="N273" t="inlineStr">
+        <is>
+          <t>Květnový 'chřestový' detail z luční rostliny, která se dnes téměř vůbec nečte jako kuchyňská.</t>
+        </is>
+      </c>
+      <c r="O273" t="inlineStr">
+        <is>
+          <t>jemně nasládlý, zeleninový</t>
+        </is>
+      </c>
+      <c r="P273" t="inlineStr">
+        <is>
+          <t>slabě bylinný</t>
+        </is>
+      </c>
+      <c r="Q273" t="inlineStr">
+        <is>
+          <t>neaplikovatelné</t>
+        </is>
+      </c>
+      <c r="R273" t="inlineStr">
+        <is>
+          <t>Používat jen mladé stonky a poupata; starší části rychle dřevnatí a kvalita jde dolů.</t>
+        </is>
+      </c>
+      <c r="S273" t="inlineStr"/>
+      <c r="T273" t="inlineStr">
+        <is>
+          <t>Sbírat střídmě z běžných lučních porostů a nepřerušovat celé populace v době květu.</t>
+        </is>
+      </c>
+      <c r="U273" t="inlineStr">
+        <is>
+          <t>kurátorovaný botanický zdroj</t>
+        </is>
+      </c>
+      <c r="V273" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="W273" t="inlineStr">
+        <is>
+          <t>S108</t>
+        </is>
+      </c>
+      <c r="X273" t="inlineStr"/>
+      <c r="Y273" t="inlineStr">
+        <is>
+          <t>Květnové rozšíření posouvá dataset i směrem k lučním stonkovým a poupatovým jedlostem.</t>
+        </is>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" t="inlineStr">
+        <is>
+          <t>R273</t>
+        </is>
+      </c>
+      <c r="B274" t="inlineStr">
+        <is>
+          <t>Heracleum sphondylium</t>
+        </is>
+      </c>
+      <c r="C274" t="inlineStr">
+        <is>
+          <t>bolševník obecný</t>
+        </is>
+      </c>
+      <c r="D274" t="inlineStr">
+        <is>
+          <t>původní, běžný</t>
+        </is>
+      </c>
+      <c r="E274" t="inlineStr">
+        <is>
+          <t>mladé stonky, řapíky a výhonky</t>
+        </is>
+      </c>
+      <c r="F274" t="inlineStr">
+        <is>
+          <t>potrava</t>
+        </is>
+      </c>
+      <c r="G274" t="inlineStr">
+        <is>
+          <t>mladé stonky a výhonky vařené jako zelenina</t>
+        </is>
+      </c>
+      <c r="H274" t="inlineStr">
+        <is>
+          <t>téměř zapomenuté</t>
+        </is>
+      </c>
+      <c r="I274" t="inlineStr">
+        <is>
+          <t>nízká až střední</t>
+        </is>
+      </c>
+      <c r="J274" t="inlineStr">
+        <is>
+          <t>vlhčí louky, příkopy, lemy cest, křoviny a lesní okraje</t>
+        </is>
+      </c>
+      <c r="K274" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="L274" t="inlineStr">
+        <is>
+          <t>úplně mladé výhonky a stonky těsně po vyrašení, před kvetením</t>
+        </is>
+      </c>
+      <c r="M274" t="inlineStr">
+        <is>
+          <t>Použitelné jsou jen mladé výhonky a stonky, ideálně po oloupání a tepelné úpravě; starší části rychle ztrácejí kvalitu.</t>
+        </is>
+      </c>
+      <c r="N274" t="inlineStr">
+        <is>
+          <t>Vysoce niche květnová zelenina pro opravdu pokročilé sběrače, historicky ceněná, dnes skoro neznámá.</t>
+        </is>
+      </c>
+      <c r="O274" t="inlineStr">
+        <is>
+          <t>výrazně zeleninový, lehce aromatický</t>
+        </is>
+      </c>
+      <c r="P274" t="inlineStr">
+        <is>
+          <t>miříkovitý, kořenitý</t>
+        </is>
+      </c>
+      <c r="Q274" t="inlineStr">
+        <is>
+          <t>neaplikovatelné</t>
+        </is>
+      </c>
+      <c r="R274" t="inlineStr">
+        <is>
+          <t>Fototoxicita a riziko záměny s jinými miříkovitými včetně nebezpečných druhů; bez naprosté jistoty určování a ochrany kůže nesbírat.</t>
+        </is>
+      </c>
+      <c r="S274" t="inlineStr">
+        <is>
+          <t>Nevhodné pro začátečníky; citlivá kůže může reagovat i na mízu.</t>
+        </is>
+      </c>
+      <c r="T274" t="inlineStr">
+        <is>
+          <t>Sbírat jen malé množství z běžných porostů a pouze tam, kde je sběr legální a nehrozí poškození citlivého stanoviště.</t>
+        </is>
+      </c>
+      <c r="U274" t="inlineStr">
+        <is>
+          <t>kurátorovaný botanický zdroj</t>
+        </is>
+      </c>
+      <c r="V274" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="W274" t="inlineStr">
+        <is>
+          <t>S109</t>
+        </is>
+      </c>
+      <c r="X274" t="inlineStr"/>
+      <c r="Y274" t="inlineStr">
+        <is>
+          <t>Zařazeno záměrně jako 'tajná' květnová rostlina, ale s nejostřejším bezpečnostním rámcem z celé vlny.</t>
         </is>
       </c>
     </row>
@@ -32588,7 +34629,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D96"/>
+  <dimension ref="A1:D110"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -34706,6 +36747,314 @@
       <c r="D96" t="inlineStr">
         <is>
           <t>Kurátorovaný zdroj pro zvonek kopřivolistý jako regionálně doloženou, ale okrajovou listovou zeleninu.</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>S96</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>PFAF: Tussilago farfara</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>https://pfaf.org/user/Plant.aspx?LatinName=Tussilago+farfara</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>Kurátorovaný zdroj pro časné jarní květní využití podbělu a opatrné použití na čaj se silným upozorněním na pyrrolizidinové alkaloidy.</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>S97</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>PFAF: Primula veris</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>https://pfaf.org/user/Plant.aspx?LatinName=Primula_veris</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>Kurátorovaný zdroj pro prvosenku jarní: časné listy, květy, konzervy i jarní květní nápoje.</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>S98</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>PFAF: Primula elatior</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>https://pfaf.org/User/Plant.aspx?LatinName=Primula+elatior</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>Kurátorovaný zdroj pro prvosenku vyšší jako velmi ranou lesní listovou zeleninu.</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>S99</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>PFAF: Lamium purpureum</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>https://pfaf.org/user/Plant.aspx?LatinName=Lamium_purpureum</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>Kurátorovaný zdroj pro hluchavku nachovou jako nenápadnou, ale dobře dostupnou předjarní zeleň.</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>S100</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>PFAF: Lamium album</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>https://pfaf.org/user/plant.aspx?latinname=Lamium+album</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>Kurátorovaný zdroj pro hluchavku bílou: mladé listy i sušené květy na jemný čaj.</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>S101</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>PFAF: Alliaria petiolata</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>https://pfaf.org/user/Plant.aspx?LatinName=alliaria+petiolata</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>Kurátorovaný zdroj pro česnáček lékařský včetně listů, květů a mladých šešulek.</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>S102</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>PFAF: Robinia pseudoacacia</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>https://pfaf.org/user/Plant.aspx?LatinName=robinia_pseudoacacia</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>Kurátorovaný zdroj pro květy akátu/trnovníku akátu; zároveň zdůrazňuje nutnost opatrnosti, protože ostatní části rostliny jsou toxické.</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>S103</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>PFAF: Humulus lupulus</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>https://pfaf.org/user/plant.aspx?latinname=Humulus+lupulus</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>Kurátorovaný zdroj pro jarní chmelové výhonky a listy, využitelné jen v krátkém květnovém okně.</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>S104</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>PFAF: Epilobium angustifolium</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>https://pfaf.org/user/Plant.aspx?LatinName=Epilobium+angustifolium</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>Kurátorovaný zdroj pro vrbovku úzkolistou jako jarní výhonkovou zeleninu i čajovou rostlinu.</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>S105</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>UAF Extension: Fireweed</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>https://www.uaf.edu/ces/publications/database/food/files/pdfs/FNH-00106-Fireweed-02-23-24.pdf</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>Aljašský extension materiál s praktickými recepty na výhonky, želé, čaj a ledničkové pickles z vrbovky úzkolisté.</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>S106</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>Luke / SPECICROP: fermentation of fireweed</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>https://www.agrowebcee.net/uploads/media/luke-luobio_72_2016.pdf</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>Finsko-ruský technický materiál k tradiční i poloprůmyslové fermentaci Epilobium angustifolium pro Ivan čaj.</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>S107</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>PFAF: Silene vulgaris</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>https://pfaf.org/user/Plant.aspx?LatinName=Silene_vulgaris</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>Kurátorovaný zdroj pro silenku nadmutou jako výrazně ne-mainstreamovou evropskou jarní zeleninu.</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>S108</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>PFAF: Tragopogon pratensis</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>https://pfaf.org/user/Plant.aspx?LatinName=Tragopogon+pratensis</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>Kurátorovaný zdroj pro kozí bradu luční včetně stonků a poupat podávaných jako 'divoký chřest'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>S109</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>PFAF: Heracleum sphondylium</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>https://pfaf.org/user/Plant.aspx?LatinName=Heracleum+Sphondylium</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>Kurátorovaný zdroj pro bolševník obecný; použitelné jen s výrazným varováním kvůli fototoxicitě a záměně s jinými miříkovitými.</t>
         </is>
       </c>
     </row>
@@ -34720,7 +37069,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K87"/>
+  <dimension ref="A1:K92"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -39692,6 +42041,291 @@
       <c r="K87" t="inlineStr">
         <is>
           <t>Po důkladném odpaření plnit horké do čistých lahví a skladovat v chladu a temnu.</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>R258</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>podběl lékařský</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>Tussilago farfara</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>pití</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>sušené listy a květy na občasný nálev</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>listy a květy</t>
+        </is>
+      </c>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>III–V + sušení</t>
+        </is>
+      </c>
+      <c r="H88" t="inlineStr">
+        <is>
+          <t>jílovité náspy, okraje cest, výsypky, rumiště, vlhčí svahy a narušené půdy</t>
+        </is>
+      </c>
+      <c r="I88" t="inlineStr">
+        <is>
+          <t>sušení na čaj</t>
+        </is>
+      </c>
+      <c r="J88" t="inlineStr">
+        <is>
+          <t>cca 6–12 měsíců</t>
+        </is>
+      </c>
+      <c r="K88" t="inlineStr">
+        <is>
+          <t>Sušit rychle v tenké vrstvě, skladovat v suchu a temnu. Kvůli alkaloidům jen střídmé a občasné použití.</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>R261</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>prvosenka jarní</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>Primula veris</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>potrava</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>květy do salátu / ozdoby / konzervy</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>květy</t>
+        </is>
+      </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>IV–V</t>
+        </is>
+      </c>
+      <c r="H89" t="inlineStr">
+        <is>
+          <t>světlejší louky, remízky, okraje lesů, suché až mezofilní trávníky</t>
+        </is>
+      </c>
+      <c r="I89" t="inlineStr">
+        <is>
+          <t>zavařenina / květní konzerva</t>
+        </is>
+      </c>
+      <c r="J89" t="inlineStr">
+        <is>
+          <t>cca 6–12 měsíců</t>
+        </is>
+      </c>
+      <c r="K89" t="inlineStr">
+        <is>
+          <t>Zpracovat jen čisté květy bez stopek; po otevření uchovávat v chladu.</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>R264</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>hluchavka bílá</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>Lamium album</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>pití</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>sušené květy na jemný čaj</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>květy</t>
+        </is>
+      </c>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>V–IX + sušení</t>
+        </is>
+      </c>
+      <c r="H90" t="inlineStr">
+        <is>
+          <t>živé ploty, křoviny, lemy cest, zahrady a ruderální okraje</t>
+        </is>
+      </c>
+      <c r="I90" t="inlineStr">
+        <is>
+          <t>sušení na čaj</t>
+        </is>
+      </c>
+      <c r="J90" t="inlineStr">
+        <is>
+          <t>cca 6–12 měsíců</t>
+        </is>
+      </c>
+      <c r="K90" t="inlineStr">
+        <is>
+          <t>Sušit v tenké vrstvě a chránit před zapařením. Uchovávat v uzavřené nádobě a temnu.</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>R267</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>trnovník akát</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>Robinia pseudoacacia</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>potrava</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>květy vařené / nápoj / zavařenina</t>
+        </is>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>květy</t>
+        </is>
+      </c>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>V–VI</t>
+        </is>
+      </c>
+      <c r="H91" t="inlineStr">
+        <is>
+          <t>teplejší stráně, aleje, remízky, suché meze, městské a příměstské výsadby</t>
+        </is>
+      </c>
+      <c r="I91" t="inlineStr">
+        <is>
+          <t>sirup / zavařenina</t>
+        </is>
+      </c>
+      <c r="J91" t="inlineStr">
+        <is>
+          <t>cca 6–12 měsíců</t>
+        </is>
+      </c>
+      <c r="K91" t="inlineStr">
+        <is>
+          <t>Zpracovat jen samotné květy bez zelených částí; po otevření skladovat v chladu a vždy hlídat čistotu suroviny.</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>R270</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>vrbovka úzkolistá</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>Epilobium angustifolium</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>pití</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>fermentované a sušené listy na Ivan čaj</t>
+        </is>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>mladé listy a vrcholky</t>
+        </is>
+      </c>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>V–VIII + fermentace + sušení</t>
+        </is>
+      </c>
+      <c r="H92" t="inlineStr">
+        <is>
+          <t>světliny, paseky, náspy, horské a podhorské disturbované lokality</t>
+        </is>
+      </c>
+      <c r="I92" t="inlineStr">
+        <is>
+          <t>fermentace + sušení</t>
+        </is>
+      </c>
+      <c r="J92" t="inlineStr">
+        <is>
+          <t>cca 6–18 měsíců</t>
+        </is>
+      </c>
+      <c r="K92" t="inlineStr">
+        <is>
+          <t>Po fermentaci důkladně dosušit, jinak hrozí plesnivění. Uchovávat v suchu, temnu a těsné nádobě.</t>
         </is>
       </c>
     </row>

</xml_diff>